<commit_message>
Corrige o nome do autor nos robôs, planilha e README
Claude-Session: https://claude.ai/code/session_01WggAWLjcJSto6UsG59pmDJ
</commit_message>
<xml_diff>
--- a/controle_equipamentos.xlsx
+++ b/controle_equipamentos.xlsx
@@ -1070,7 +1070,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Lucas Faria  |  Matrícula cbk3574  |  github.com/lucasdpr/controle-equipamentos</t>
+          <t>Lucas Gabriel de Paula Rafael  |  Matrícula cbk3574  |  github.com/lucasdpr/controle-equipamentos</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>Autor: Lucas Faria  |  Matrícula cbk3574  |  github.com/lucasdpr/controle-equipamentos</t>
+          <t>Autor: Lucas Gabriel de Paula Rafael  |  Matrícula cbk3574  |  github.com/lucasdpr/controle-equipamentos</t>
         </is>
       </c>
     </row>

</xml_diff>